<commit_message>
Reports: July 2026 H1 (1 report(s))
</commit_message>
<xml_diff>
--- a/Payroll Report/Payroll_Report_July_2026_H1.xlsx
+++ b/Payroll Report/Payroll_Report_July_2026_H1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t>Employee</t>
   </si>
@@ -90,16 +90,10 @@
     <t>July 2026 H1  (2026-07-01 to 2026-07-14 inclusive)</t>
   </si>
   <si>
-    <t>Run date (UTC)</t>
-  </si>
-  <si>
-    <t>2026-07-16</t>
-  </si>
-  <si>
     <t>Generated (UTC)</t>
   </si>
   <si>
-    <t>2026-07-16 07:14:31</t>
+    <t>2026-07-16 09:59:51</t>
   </si>
   <si>
     <t>Source</t>
@@ -409,7 +403,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="18.484375" customWidth="true" bestFit="true"/>
@@ -472,14 +466,6 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>36</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Reports: July 2026 H1 (6 report(s))
</commit_message>
<xml_diff>
--- a/Payroll Report/Payroll_Report_July_2026_H1.xlsx
+++ b/Payroll Report/Payroll_Report_July_2026_H1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="70">
   <si>
     <t>Employee</t>
   </si>
@@ -39,40 +39,145 @@
     <t>Pay</t>
   </si>
   <si>
+    <t>EM0015</t>
+  </si>
+  <si>
+    <t>Melissa Green</t>
+  </si>
+  <si>
+    <t>EM0019</t>
+  </si>
+  <si>
+    <t>Michelle Murphy</t>
+  </si>
+  <si>
+    <t>Supervisor</t>
+  </si>
+  <si>
+    <t>EM0009</t>
+  </si>
+  <si>
+    <t>Nancy Lee</t>
+  </si>
+  <si>
+    <t>EM0028</t>
+  </si>
+  <si>
+    <t>Ronald Carter</t>
+  </si>
+  <si>
+    <t>EM0014</t>
+  </si>
+  <si>
+    <t>Dorothy Rogers</t>
+  </si>
+  <si>
+    <t>EM0024</t>
+  </si>
+  <si>
+    <t>Brian Rogers</t>
+  </si>
+  <si>
+    <t>EM0006</t>
+  </si>
+  <si>
+    <t>Helen Stewart</t>
+  </si>
+  <si>
+    <t>EM0026</t>
+  </si>
+  <si>
+    <t>Jason Collins</t>
+  </si>
+  <si>
+    <t>EM0021</t>
+  </si>
+  <si>
+    <t>Laura Ross</t>
+  </si>
+  <si>
+    <t>EM0025</t>
+  </si>
+  <si>
+    <t>Amy Price</t>
+  </si>
+  <si>
+    <t>EM0010</t>
+  </si>
+  <si>
+    <t>Pamela Garcia</t>
+  </si>
+  <si>
+    <t>EM0022</t>
+  </si>
+  <si>
+    <t>Kevin Harris</t>
+  </si>
+  <si>
+    <t>EM0002</t>
+  </si>
+  <si>
+    <t>Robert King</t>
+  </si>
+  <si>
+    <t>EM0016</t>
+  </si>
+  <si>
+    <t>Matthew Reed</t>
+  </si>
+  <si>
+    <t>EM0011</t>
+  </si>
+  <si>
+    <t>Stephanie Baker</t>
+  </si>
+  <si>
+    <t>EM0004</t>
+  </si>
+  <si>
+    <t>Christopher Bryant</t>
+  </si>
+  <si>
+    <t>EM0007</t>
+  </si>
+  <si>
+    <t>Brenda Allen</t>
+  </si>
+  <si>
     <t>EM0013</t>
   </si>
   <si>
-    <t>Carol Stewart</t>
-  </si>
-  <si>
-    <t>EM0010</t>
-  </si>
-  <si>
-    <t>Pamela Garcia</t>
-  </si>
-  <si>
-    <t>EM0009</t>
-  </si>
-  <si>
-    <t>Nancy Johnson</t>
-  </si>
-  <si>
-    <t>EM0017</t>
-  </si>
-  <si>
-    <t>Matthew Carter</t>
+    <t>Steven Martin</t>
+  </si>
+  <si>
+    <t>EM0029</t>
+  </si>
+  <si>
+    <t>Rachel Bell</t>
+  </si>
+  <si>
+    <t>EM0023</t>
+  </si>
+  <si>
+    <t>Sharon Morris</t>
+  </si>
+  <si>
+    <t>EM0003</t>
+  </si>
+  <si>
+    <t>Richard Foster</t>
+  </si>
+  <si>
+    <t>EM0020</t>
+  </si>
+  <si>
+    <t>Anthony Ward</t>
   </si>
   <si>
     <t>EM0012</t>
   </si>
   <si>
-    <t>Stephanie Morris</t>
-  </si>
-  <si>
-    <t>EM0011</t>
-  </si>
-  <si>
-    <t>Pamela Parker</t>
+    <t>Carol Murray</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -93,7 +198,7 @@
     <t>Generated (UTC)</t>
   </si>
   <si>
-    <t>2026-07-16 15:22:29</t>
+    <t>2026-07-23 07:38:06</t>
   </si>
   <si>
     <t>Source</t>
@@ -105,19 +210,19 @@
     <t>Basis</t>
   </si>
   <si>
-    <t>Job assignments completed within the period (jobassign_status = 'C')</t>
+    <t>Jobs completed within the period (status = 'C'), keyed on updated_at</t>
   </si>
   <si>
     <t>Formula</t>
   </si>
   <si>
-    <t>Pay = SUM(jobassign_hours) x emp_hourly_rate</t>
+    <t>Pay = SUM(hours) x emp_hourly_rate</t>
   </si>
   <si>
     <t>Technicians paid</t>
   </si>
   <si>
-    <t>6</t>
+    <t>23</t>
   </si>
 </sst>
 </file>
@@ -187,17 +292,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.23046875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="16.5625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="18.4375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.9375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.421875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="5.53125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="7.28125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="8.26171875" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="15.76953125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="11.51171875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="12.78515625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -237,19 +342,19 @@
         <v>1</v>
       </c>
       <c r="D2" t="n" s="2">
-        <v>1364.81</v>
+        <v>1699.4</v>
       </c>
       <c r="E2" t="n" s="0">
-        <v>1.0</v>
+        <v>7.0</v>
       </c>
       <c r="F2" t="n" s="2">
-        <v>8.89</v>
+        <v>22.27</v>
       </c>
       <c r="G2" t="n" s="2">
-        <v>8.89</v>
+        <v>3.18</v>
       </c>
       <c r="H2" t="n" s="2">
-        <v>12133.1609</v>
+        <v>37845.638</v>
       </c>
     </row>
     <row r="3">
@@ -260,140 +365,582 @@
         <v>11</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n" s="2">
-        <v>1945.93</v>
+        <v>2977.2</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="F3" t="n" s="2">
-        <v>6.11</v>
+        <v>9.3</v>
       </c>
       <c r="G3" t="n" s="2">
-        <v>6.11</v>
+        <v>3.1</v>
       </c>
       <c r="H3" t="n" s="2">
-        <v>11889.6323</v>
+        <v>27687.96</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>1</v>
       </c>
       <c r="D4" t="n" s="2">
-        <v>1404.6</v>
+        <v>1909.13</v>
       </c>
       <c r="E4" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F4" t="n" s="2">
-        <v>6.86</v>
+        <v>13.72</v>
       </c>
       <c r="G4" t="n" s="2">
-        <v>3.43</v>
+        <v>4.57</v>
       </c>
       <c r="H4" t="n" s="2">
-        <v>9635.556</v>
+        <v>26193.2636</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D5" t="n" s="2">
-        <v>1509.04</v>
+        <v>3162.79</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="F5" t="n" s="2">
-        <v>5.42</v>
+        <v>8.16</v>
       </c>
       <c r="G5" t="n" s="2">
-        <v>5.42</v>
+        <v>2.72</v>
       </c>
       <c r="H5" t="n" s="2">
-        <v>8178.9968</v>
+        <v>25808.3664</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>1</v>
       </c>
       <c r="D6" t="n" s="2">
-        <v>1355.87</v>
+        <v>1861.37</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="F6" t="n" s="2">
-        <v>4.7</v>
+        <v>13.4</v>
       </c>
       <c r="G6" t="n" s="2">
-        <v>4.7</v>
+        <v>4.47</v>
       </c>
       <c r="H6" t="n" s="2">
-        <v>6372.589</v>
+        <v>24942.358</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>1</v>
       </c>
       <c r="D7" t="n" s="2">
-        <v>2073.5</v>
+        <v>2218.49</v>
       </c>
       <c r="E7" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="F7" t="n" s="2">
+        <v>10.5</v>
+      </c>
+      <c r="G7" t="n" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="H7" t="n" s="2">
+        <v>23294.145</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n" s="2">
+        <v>1961.26</v>
+      </c>
+      <c r="E8" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="F8" t="n" s="2">
+        <v>11.47</v>
+      </c>
+      <c r="G8" t="n" s="2">
+        <v>2.87</v>
+      </c>
+      <c r="H8" t="n" s="2">
+        <v>22495.6522</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n" s="2">
+        <v>2246.95</v>
+      </c>
+      <c r="E9" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="F9" t="n" s="2">
+        <v>9.87</v>
+      </c>
+      <c r="G9" t="n" s="2">
+        <v>3.29</v>
+      </c>
+      <c r="H9" t="n" s="2">
+        <v>22177.3965</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n" s="2">
+        <v>1563.39</v>
+      </c>
+      <c r="E10" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="F10" t="n" s="2">
+        <v>14.12</v>
+      </c>
+      <c r="G10" t="n" s="2">
+        <v>2.82</v>
+      </c>
+      <c r="H10" t="n" s="2">
+        <v>22075.0668</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n" s="2">
+        <v>2178.72</v>
+      </c>
+      <c r="E11" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="F11" t="n" s="2">
+        <v>10.12</v>
+      </c>
+      <c r="G11" t="n" s="2">
+        <v>3.37</v>
+      </c>
+      <c r="H11" t="n" s="2">
+        <v>22048.6464</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n" s="2">
+        <v>1679.46</v>
+      </c>
+      <c r="E12" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="F12" t="n" s="2">
+        <v>8.64</v>
+      </c>
+      <c r="G12" t="n" s="2">
+        <v>2.88</v>
+      </c>
+      <c r="H12" t="n" s="2">
+        <v>14510.5344</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n" s="2">
+        <v>2170.52</v>
+      </c>
+      <c r="E13" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="F13" t="n" s="2">
+        <v>6.35</v>
+      </c>
+      <c r="G13" t="n" s="2">
+        <v>3.18</v>
+      </c>
+      <c r="H13" t="n" s="2">
+        <v>13782.802</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n" s="2">
+        <v>2063.49</v>
+      </c>
+      <c r="E14" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="F14" t="n" s="2">
+        <v>6.43</v>
+      </c>
+      <c r="G14" t="n" s="2">
+        <v>3.22</v>
+      </c>
+      <c r="H14" t="n" s="2">
+        <v>13268.2407</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n" s="2">
+        <v>1347.12</v>
+      </c>
+      <c r="E15" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="F15" t="n" s="2">
+        <v>9.76</v>
+      </c>
+      <c r="G15" t="n" s="2">
+        <v>3.25</v>
+      </c>
+      <c r="H15" t="n" s="2">
+        <v>13147.8912</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n" s="2">
+        <v>1355.94</v>
+      </c>
+      <c r="E16" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="F16" t="n" s="2">
+        <v>9.54</v>
+      </c>
+      <c r="G16" t="n" s="2">
+        <v>4.77</v>
+      </c>
+      <c r="H16" t="n" s="2">
+        <v>12935.6676</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n" s="2">
+        <v>1424.83</v>
+      </c>
+      <c r="E17" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="F17" t="n" s="2">
+        <v>7.99</v>
+      </c>
+      <c r="G17" t="n" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="H17" t="n" s="2">
+        <v>11384.3917</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n" s="2">
+        <v>1680.13</v>
+      </c>
+      <c r="E18" t="n" s="0">
         <v>1.0</v>
       </c>
-      <c r="F7" t="n" s="2">
-        <v>2.52</v>
-      </c>
-      <c r="G7" t="n" s="2">
-        <v>2.52</v>
-      </c>
-      <c r="H7" t="n" s="2">
-        <v>5225.22</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="4">
-        <v>20</v>
-      </c>
-      <c r="E8" t="n" s="4">
-        <v>7.0</v>
-      </c>
-      <c r="F8" t="n" s="3">
-        <v>34.5</v>
-      </c>
-      <c r="H8" t="n" s="3">
-        <v>53435.155</v>
+      <c r="F18" t="n" s="2">
+        <v>5.6</v>
+      </c>
+      <c r="G18" t="n" s="2">
+        <v>5.6</v>
+      </c>
+      <c r="H18" t="n" s="2">
+        <v>9408.728</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n" s="2">
+        <v>2214.55</v>
+      </c>
+      <c r="E19" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F19" t="n" s="2">
+        <v>3.71</v>
+      </c>
+      <c r="G19" t="n" s="2">
+        <v>3.71</v>
+      </c>
+      <c r="H19" t="n" s="2">
+        <v>8215.9805</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n" s="2">
+        <v>2228.91</v>
+      </c>
+      <c r="E20" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="F20" t="n" s="2">
+        <v>3.61</v>
+      </c>
+      <c r="G20" t="n" s="2">
+        <v>1.81</v>
+      </c>
+      <c r="H20" t="n" s="2">
+        <v>8046.3651</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n" s="2">
+        <v>1452.84</v>
+      </c>
+      <c r="E21" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F21" t="n" s="2">
+        <v>5.23</v>
+      </c>
+      <c r="G21" t="n" s="2">
+        <v>5.23</v>
+      </c>
+      <c r="H21" t="n" s="2">
+        <v>7598.3532</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n" s="2">
+        <v>1643.96</v>
+      </c>
+      <c r="E22" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F22" t="n" s="2">
+        <v>3.48</v>
+      </c>
+      <c r="G22" t="n" s="2">
+        <v>3.48</v>
+      </c>
+      <c r="H22" t="n" s="2">
+        <v>5720.9808</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n" s="2">
+        <v>1734.77</v>
+      </c>
+      <c r="E23" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F23" t="n" s="2">
+        <v>1.79</v>
+      </c>
+      <c r="G23" t="n" s="2">
+        <v>1.79</v>
+      </c>
+      <c r="H23" t="n" s="2">
+        <v>3105.2383</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n" s="2">
+        <v>1510.98</v>
+      </c>
+      <c r="E24" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F24" t="n" s="2">
+        <v>1.84</v>
+      </c>
+      <c r="G24" t="n" s="2">
+        <v>1.84</v>
+      </c>
+      <c r="H24" t="n" s="2">
+        <v>2780.2032</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="4">
+        <v>55</v>
+      </c>
+      <c r="E25" t="n" s="4">
+        <v>59.0</v>
+      </c>
+      <c r="F25" t="n" s="3">
+        <v>196.9</v>
+      </c>
+      <c r="H25" t="n" s="3">
+        <v>378473.8696000001</v>
       </c>
     </row>
   </sheetData>
@@ -407,63 +954,63 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="18.484375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="64.7578125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="64.4921875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>22</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="1">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>24</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="1">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>26</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>28</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="1">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>30</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="1">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>32</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="1">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>34</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>